<commit_message>
Added codes for Brazil, Chile and Turkey
</commit_message>
<xml_diff>
--- a/data/xlsx/metadata.xlsx
+++ b/data/xlsx/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mark/sites/codeforiati/gov-id-finder-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77890723-856B-334C-BC61-3AD96F1845B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71858CA7-390A-E648-9CA2-8F9E5EA0ECDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44940" yWindow="-2080" windowWidth="22260" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="44940" yWindow="-1360" windowWidth="22260" windowHeight="16560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="195">
   <si>
     <t>Country_name</t>
   </si>
@@ -592,6 +592,33 @@
   <si>
     <t>https://www.finances.gov.ma/Publication/db/2023/BO_7259-bis_fr.pdf</t>
   </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>https://www.tesourotransparente.gov.br/ckan/dataset/lista-de-orgaos-do-siafi</t>
+  </si>
+  <si>
+    <t>CL</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>https://www.dipres.gob.cl/597/w3-multipropertyvalues-15145-37782.html</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>https://www.sbb.gov.tr/butce-cagrisi-ve-butce-hazirlama-rehberleri/#1631294260433-cce691d9-4a8c</t>
+  </si>
 </sst>
 </file>
 
@@ -917,7 +944,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1003"/>
+  <dimension ref="A1:AA1006"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="74.83203125" customWidth="1"/>
@@ -1257,17 +1284,17 @@
       <c r="AA9" s="1"/>
     </row>
     <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>147</v>
+      <c r="A10" s="5" t="s">
+        <v>187</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>148</v>
+      <c r="B10" s="8" t="s">
+        <v>186</v>
       </c>
-      <c r="C10" t="s">
-        <v>146</v>
+      <c r="C10" s="1">
+        <v>2026</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>149</v>
+      <c r="D10" s="4" t="s">
+        <v>188</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1295,16 +1322,16 @@
     </row>
     <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>147</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>115</v>
+      <c r="B11" s="9" t="s">
+        <v>148</v>
       </c>
-      <c r="C11" s="1">
-        <v>2020</v>
+      <c r="C11" t="s">
+        <v>146</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>13</v>
+      <c r="D11" s="6" t="s">
+        <v>149</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1332,16 +1359,16 @@
     </row>
     <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C12" s="1">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -1368,17 +1395,17 @@
       <c r="AA12" s="1"/>
     </row>
     <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="5" t="s">
-        <v>162</v>
+      <c r="A13" t="s">
+        <v>55</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>163</v>
+        <v>116</v>
       </c>
       <c r="C13" s="1">
-        <v>2024</v>
+        <v>2019</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>164</v>
+      <c r="D13" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -1405,17 +1432,17 @@
       <c r="AA13" s="1"/>
     </row>
     <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" t="s">
-        <v>56</v>
+      <c r="A14" s="5" t="s">
+        <v>162</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="C14" s="1">
         <v>2024</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -1443,16 +1470,16 @@
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>11</v>
+        <v>117</v>
       </c>
       <c r="C15" s="1">
         <v>2024</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1479,17 +1506,17 @@
       <c r="AA15" s="1"/>
     </row>
     <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" t="s">
-        <v>58</v>
+      <c r="A16" s="5" t="s">
+        <v>189</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>118</v>
+        <v>190</v>
       </c>
       <c r="C16" s="1">
-        <v>2019</v>
+        <v>2026</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>14</v>
+      <c r="D16" s="4" t="s">
+        <v>191</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -1517,16 +1544,16 @@
     </row>
     <row r="17" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="C17" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1554,16 +1581,16 @@
     </row>
     <row r="18" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C18" s="1">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -1591,16 +1618,16 @@
     </row>
     <row r="19" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C19" s="1">
-        <v>2017</v>
+        <v>2023</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>16</v>
+      <c r="D19" s="4" t="s">
+        <v>171</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -1627,17 +1654,17 @@
       <c r="AA19" s="1"/>
     </row>
     <row r="20" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="5" t="s">
-        <v>168</v>
+      <c r="A20" t="s">
+        <v>59</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>169</v>
+        <v>120</v>
       </c>
       <c r="C20" s="1">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>170</v>
+        <v>15</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1665,16 +1692,16 @@
     </row>
     <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C21" s="1">
-        <v>2024</v>
+        <v>2017</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>182</v>
+      <c r="D21" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -1701,17 +1728,17 @@
       <c r="AA21" s="1"/>
     </row>
     <row r="22" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" t="s">
-        <v>95</v>
+      <c r="A22" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>123</v>
+        <v>169</v>
       </c>
       <c r="C22" s="1">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>45</v>
+        <v>170</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -1739,16 +1766,16 @@
     </row>
     <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
-      <c r="B23" s="10" t="s">
-        <v>101</v>
+      <c r="B23" s="8" t="s">
+        <v>122</v>
       </c>
-      <c r="C23">
-        <v>2012</v>
+      <c r="C23" s="1">
+        <v>2024</v>
       </c>
-      <c r="D23" t="s">
-        <v>102</v>
+      <c r="D23" s="4" t="s">
+        <v>182</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1776,16 +1803,16 @@
     </row>
     <row r="24" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C24" s="1">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -1813,16 +1840,16 @@
     </row>
     <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>125</v>
+      <c r="B25" s="10" t="s">
+        <v>101</v>
       </c>
-      <c r="C25" s="1">
-        <v>2019</v>
+      <c r="C25">
+        <v>2012</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>17</v>
+      <c r="D25" t="s">
+        <v>102</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -1850,16 +1877,16 @@
     </row>
     <row r="26" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>150</v>
+      <c r="C26" s="1">
+        <v>2018</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>109</v>
+      <c r="D26" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1887,16 +1914,16 @@
     </row>
     <row r="27" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C27" s="1">
-        <v>2020</v>
+        <v>2019</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>18</v>
+      <c r="D27" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -1924,16 +1951,16 @@
     </row>
     <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
-      <c r="C28" s="1">
-        <v>2021</v>
+      <c r="C28" s="1" t="s">
+        <v>150</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>36</v>
+      <c r="D28" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -1961,16 +1988,16 @@
     </row>
     <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>64</v>
       </c>
-      <c r="B29" s="10" t="s">
-        <v>103</v>
+      <c r="B29" s="8" t="s">
+        <v>127</v>
       </c>
-      <c r="C29">
-        <v>2019</v>
+      <c r="C29" s="1">
+        <v>2020</v>
       </c>
-      <c r="D29" t="s">
-        <v>104</v>
+      <c r="D29" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -1998,16 +2025,16 @@
     </row>
     <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C30" s="1">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>184</v>
+        <v>36</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -2035,16 +2062,16 @@
     </row>
     <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>130</v>
+      <c r="B31" s="10" t="s">
+        <v>103</v>
       </c>
-      <c r="C31" s="1">
-        <v>2021</v>
+      <c r="C31">
+        <v>2019</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>19</v>
+      <c r="D31" t="s">
+        <v>104</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -2071,17 +2098,17 @@
       <c r="AA31" s="1"/>
     </row>
     <row r="32" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="5" t="s">
-        <v>151</v>
+      <c r="A32" t="s">
+        <v>66</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="C32" s="1">
         <v>2024</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>185</v>
+      <c r="D32" s="2" t="s">
+        <v>184</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -2109,16 +2136,16 @@
     </row>
     <row r="33" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C33" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>110</v>
+      <c r="D33" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -2145,17 +2172,17 @@
       <c r="AA33" s="1"/>
     </row>
     <row r="34" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" t="s">
-        <v>69</v>
+      <c r="A34" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>21</v>
+        <v>152</v>
       </c>
       <c r="C34" s="1">
         <v>2024</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>172</v>
+      <c r="D34" s="4" t="s">
+        <v>185</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -2183,16 +2210,16 @@
     </row>
     <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C35" s="1">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -2220,16 +2247,16 @@
     </row>
     <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C36" s="1">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>23</v>
+        <v>172</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -2257,16 +2284,16 @@
     </row>
     <row r="37" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C37" s="1">
-        <v>2021</v>
+        <v>2017</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>20</v>
+      <c r="D37" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -2294,16 +2321,16 @@
     </row>
     <row r="38" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>134</v>
+        <v>22</v>
       </c>
       <c r="C38" s="1">
         <v>2020</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -2330,17 +2357,17 @@
       <c r="AA38" s="1"/>
     </row>
     <row r="39" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="5" t="s">
-        <v>165</v>
+      <c r="A39" t="s">
+        <v>68</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>166</v>
+        <v>133</v>
       </c>
       <c r="C39" s="1">
-        <v>2024</v>
+        <v>2021</v>
       </c>
-      <c r="D39" s="4" t="s">
-        <v>167</v>
+      <c r="D39" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -2368,16 +2395,16 @@
     </row>
     <row r="40" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C40" s="1">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>173</v>
+        <v>24</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
@@ -2405,16 +2432,16 @@
     </row>
     <row r="41" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="5" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="C41" s="1">
         <v>2024</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -2442,16 +2469,16 @@
     </row>
     <row r="42" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C42" s="1">
-        <v>2019</v>
+        <v>2023</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>28</v>
+      <c r="D42" s="3" t="s">
+        <v>173</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -2478,17 +2505,17 @@
       <c r="AA42" s="1"/>
     </row>
     <row r="43" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" t="s">
-        <v>74</v>
+      <c r="A43" s="5" t="s">
+        <v>153</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="C43" s="1">
-        <v>2021</v>
+        <v>2024</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>27</v>
+      <c r="D43" s="4" t="s">
+        <v>155</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -2516,16 +2543,16 @@
     </row>
     <row r="44" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>25</v>
+      <c r="B44" s="8" t="s">
+        <v>136</v>
       </c>
       <c r="C44" s="1">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -2553,16 +2580,16 @@
     </row>
     <row r="45" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C45" s="1">
         <v>2021</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -2589,17 +2616,17 @@
       <c r="AA45" s="1"/>
     </row>
     <row r="46" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A46" s="5" t="s">
-        <v>79</v>
+      <c r="A46" t="s">
+        <v>73</v>
       </c>
-      <c r="B46" s="10" t="s">
-        <v>105</v>
+      <c r="B46" s="7" t="s">
+        <v>25</v>
       </c>
-      <c r="C46">
-        <v>2022</v>
+      <c r="C46" s="1">
+        <v>2021</v>
       </c>
-      <c r="D46" t="s">
-        <v>106</v>
+      <c r="D46" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -2627,16 +2654,16 @@
     </row>
     <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C47" s="1">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -2663,17 +2690,17 @@
       <c r="AA47" s="1"/>
     </row>
     <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A48" t="s">
-        <v>80</v>
+      <c r="A48" s="5" t="s">
+        <v>79</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>140</v>
+      <c r="B48" s="10" t="s">
+        <v>105</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>146</v>
+      <c r="C48">
+        <v>2022</v>
       </c>
-      <c r="D48" s="4" t="s">
-        <v>174</v>
+      <c r="D48" t="s">
+        <v>106</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -2701,16 +2728,16 @@
     </row>
     <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>33</v>
+        <v>139</v>
       </c>
       <c r="C49" s="1">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -2738,16 +2765,16 @@
     </row>
     <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
-      <c r="C50" s="1">
-        <v>2022</v>
+      <c r="C50" s="1" t="s">
+        <v>146</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>44</v>
+      <c r="D50" s="4" t="s">
+        <v>174</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -2773,18 +2800,18 @@
       <c r="Z50" s="1"/>
       <c r="AA50" s="1"/>
     </row>
-    <row r="51" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C51" s="1">
         <v>2020</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -2810,18 +2837,18 @@
       <c r="Z51" s="1"/>
       <c r="AA51" s="1"/>
     </row>
-    <row r="52" spans="1:27" ht="28" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C52" s="1">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -2848,17 +2875,17 @@
       <c r="AA52" s="1"/>
     </row>
     <row r="53" spans="1:27" ht="14" x14ac:dyDescent="0.15">
-      <c r="A53" s="5" t="s">
-        <v>156</v>
+      <c r="A53" t="s">
+        <v>81</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>157</v>
+        <v>31</v>
       </c>
       <c r="C53" s="1">
-        <v>2024</v>
+        <v>2020</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>158</v>
+      <c r="D53" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -2884,18 +2911,18 @@
       <c r="Z53" s="1"/>
       <c r="AA53" s="1"/>
     </row>
-    <row r="54" spans="1:27" ht="13" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:27" ht="28" x14ac:dyDescent="0.15">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
-      <c r="B54" s="10" t="s">
-        <v>100</v>
+      <c r="B54" s="8" t="s">
+        <v>142</v>
       </c>
-      <c r="C54">
-        <v>2023</v>
+      <c r="C54" s="1">
+        <v>2020</v>
       </c>
-      <c r="D54" s="6" t="s">
-        <v>175</v>
+      <c r="D54" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
@@ -2921,18 +2948,18 @@
       <c r="Z54" s="1"/>
       <c r="AA54" s="1"/>
     </row>
-    <row r="55" spans="1:27" ht="28" x14ac:dyDescent="0.15">
-      <c r="A55" t="s">
-        <v>87</v>
+    <row r="55" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+      <c r="A55" s="5" t="s">
+        <v>156</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>39</v>
+        <v>157</v>
       </c>
       <c r="C55" s="1">
         <v>2024</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>176</v>
+      <c r="D55" s="4" t="s">
+        <v>158</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -2958,18 +2985,18 @@
       <c r="Z55" s="1"/>
       <c r="AA55" s="1"/>
     </row>
-    <row r="56" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A56" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
-      <c r="B56" s="8" t="s">
-        <v>37</v>
+      <c r="B56" s="10" t="s">
+        <v>100</v>
       </c>
-      <c r="C56" s="1">
-        <v>2018</v>
+      <c r="C56">
+        <v>2023</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>38</v>
+      <c r="D56" s="6" t="s">
+        <v>175</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -2997,16 +3024,16 @@
     </row>
     <row r="57" spans="1:27" ht="28" x14ac:dyDescent="0.15">
       <c r="A57" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>143</v>
+        <v>39</v>
       </c>
-      <c r="C57" s="1" t="s">
-        <v>146</v>
+      <c r="C57" s="1">
+        <v>2024</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>145</v>
+      <c r="D57" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -3034,16 +3061,16 @@
     </row>
     <row r="58" spans="1:27" ht="14" x14ac:dyDescent="0.15">
       <c r="A58" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
-      <c r="C58" s="1" t="s">
-        <v>146</v>
+      <c r="C58" s="1">
+        <v>2018</v>
       </c>
-      <c r="D58" s="4" t="s">
-        <v>177</v>
+      <c r="D58" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
@@ -3069,18 +3096,18 @@
       <c r="Z58" s="1"/>
       <c r="AA58" s="1"/>
     </row>
-    <row r="59" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:27" ht="28" x14ac:dyDescent="0.15">
       <c r="A59" s="5" t="s">
-        <v>159</v>
+        <v>192</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>160</v>
+        <v>193</v>
       </c>
       <c r="C59" s="1">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>161</v>
+        <v>194</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
@@ -3106,18 +3133,18 @@
       <c r="Z59" s="1"/>
       <c r="AA59" s="1"/>
     </row>
-    <row r="60" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:27" ht="28" x14ac:dyDescent="0.15">
       <c r="A60" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
-      <c r="C60" s="1">
-        <v>2024</v>
+      <c r="C60" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>178</v>
+        <v>145</v>
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
@@ -3145,16 +3172,16 @@
     </row>
     <row r="61" spans="1:27" ht="14" x14ac:dyDescent="0.15">
       <c r="A61" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
-      <c r="C61" s="1">
-        <v>2024</v>
+      <c r="C61" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
@@ -3180,10 +3207,19 @@
       <c r="Z61" s="1"/>
       <c r="AA61" s="1"/>
     </row>
-    <row r="62" spans="1:27" ht="13" x14ac:dyDescent="0.15">
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
+    <row r="62" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+      <c r="A62" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C62" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
@@ -3208,10 +3244,19 @@
       <c r="Z62" s="1"/>
       <c r="AA62" s="1"/>
     </row>
-    <row r="63" spans="1:27" ht="13" x14ac:dyDescent="0.15">
-      <c r="B63" s="1"/>
-      <c r="C63" s="1"/>
-      <c r="D63" s="1"/>
+    <row r="63" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+      <c r="A63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C63" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>178</v>
+      </c>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
@@ -3236,10 +3281,19 @@
       <c r="Z63" s="1"/>
       <c r="AA63" s="1"/>
     </row>
-    <row r="64" spans="1:27" ht="13" x14ac:dyDescent="0.15">
-      <c r="B64" s="1"/>
-      <c r="C64" s="1"/>
-      <c r="D64" s="1"/>
+    <row r="64" spans="1:27" ht="14" x14ac:dyDescent="0.15">
+      <c r="A64" t="s">
+        <v>90</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C64" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>179</v>
+      </c>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
@@ -29556,9 +29610,93 @@
       <c r="Z1003" s="1"/>
       <c r="AA1003" s="1"/>
     </row>
+    <row r="1004" spans="2:27" ht="13" x14ac:dyDescent="0.15">
+      <c r="B1004" s="1"/>
+      <c r="C1004" s="1"/>
+      <c r="D1004" s="1"/>
+      <c r="E1004" s="1"/>
+      <c r="F1004" s="1"/>
+      <c r="G1004" s="1"/>
+      <c r="H1004" s="1"/>
+      <c r="I1004" s="1"/>
+      <c r="J1004" s="1"/>
+      <c r="K1004" s="1"/>
+      <c r="L1004" s="1"/>
+      <c r="M1004" s="1"/>
+      <c r="N1004" s="1"/>
+      <c r="O1004" s="1"/>
+      <c r="P1004" s="1"/>
+      <c r="Q1004" s="1"/>
+      <c r="R1004" s="1"/>
+      <c r="S1004" s="1"/>
+      <c r="T1004" s="1"/>
+      <c r="U1004" s="1"/>
+      <c r="V1004" s="1"/>
+      <c r="W1004" s="1"/>
+      <c r="X1004" s="1"/>
+      <c r="Y1004" s="1"/>
+      <c r="Z1004" s="1"/>
+      <c r="AA1004" s="1"/>
+    </row>
+    <row r="1005" spans="2:27" ht="13" x14ac:dyDescent="0.15">
+      <c r="B1005" s="1"/>
+      <c r="C1005" s="1"/>
+      <c r="D1005" s="1"/>
+      <c r="E1005" s="1"/>
+      <c r="F1005" s="1"/>
+      <c r="G1005" s="1"/>
+      <c r="H1005" s="1"/>
+      <c r="I1005" s="1"/>
+      <c r="J1005" s="1"/>
+      <c r="K1005" s="1"/>
+      <c r="L1005" s="1"/>
+      <c r="M1005" s="1"/>
+      <c r="N1005" s="1"/>
+      <c r="O1005" s="1"/>
+      <c r="P1005" s="1"/>
+      <c r="Q1005" s="1"/>
+      <c r="R1005" s="1"/>
+      <c r="S1005" s="1"/>
+      <c r="T1005" s="1"/>
+      <c r="U1005" s="1"/>
+      <c r="V1005" s="1"/>
+      <c r="W1005" s="1"/>
+      <c r="X1005" s="1"/>
+      <c r="Y1005" s="1"/>
+      <c r="Z1005" s="1"/>
+      <c r="AA1005" s="1"/>
+    </row>
+    <row r="1006" spans="2:27" ht="13" x14ac:dyDescent="0.15">
+      <c r="B1006" s="1"/>
+      <c r="C1006" s="1"/>
+      <c r="D1006" s="1"/>
+      <c r="E1006" s="1"/>
+      <c r="F1006" s="1"/>
+      <c r="G1006" s="1"/>
+      <c r="H1006" s="1"/>
+      <c r="I1006" s="1"/>
+      <c r="J1006" s="1"/>
+      <c r="K1006" s="1"/>
+      <c r="L1006" s="1"/>
+      <c r="M1006" s="1"/>
+      <c r="N1006" s="1"/>
+      <c r="O1006" s="1"/>
+      <c r="P1006" s="1"/>
+      <c r="Q1006" s="1"/>
+      <c r="R1006" s="1"/>
+      <c r="S1006" s="1"/>
+      <c r="T1006" s="1"/>
+      <c r="U1006" s="1"/>
+      <c r="V1006" s="1"/>
+      <c r="W1006" s="1"/>
+      <c r="X1006" s="1"/>
+      <c r="Y1006" s="1"/>
+      <c r="Z1006" s="1"/>
+      <c r="AA1006" s="1"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D61">
-    <sortCondition ref="A56:A61"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D64">
+    <sortCondition ref="A58:A64"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -29567,52 +29705,55 @@
     <hyperlink ref="D8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="D5" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="D6" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="D15" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="D12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="D14" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="D16" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="D18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="D19" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="D21" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="D25" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="D26" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="D27" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="D31" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="D33" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="D37" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="D36" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="D38" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="D35" r:id="rId23" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="D44" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="D43" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="D42" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="D47" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="D45" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="D48" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="D51" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="D49" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="D52" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="D28" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="D57" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="D56" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="D58" r:id="rId36" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="D60" r:id="rId37" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="D61" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="D17" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="D24" r:id="rId40" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="D17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D18" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D20" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D21" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D27" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D28" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D29" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D33" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="D35" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="D39" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="D38" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="D40" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="D37" r:id="rId23" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="D46" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="D45" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="D44" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="D49" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="D47" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="D50" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="D53" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="D51" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="D54" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="D30" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="D60" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="D58" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="D61" r:id="rId36" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="D63" r:id="rId37" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="D64" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="D19" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="D26" r:id="rId40" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
     <hyperlink ref="D4" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="D50" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="D22" r:id="rId43" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="D52" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="D24" r:id="rId43" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
     <hyperlink ref="D7" r:id="rId44" xr:uid="{AEC54F8E-3B97-0D42-BDBF-81F51CF558FA}"/>
-    <hyperlink ref="D10" r:id="rId45" xr:uid="{531FF59E-3ED0-7647-A071-9938F307CC65}"/>
-    <hyperlink ref="D32" r:id="rId46" xr:uid="{F44184D1-3BA6-CA4D-B592-38E9B7DD9585}"/>
-    <hyperlink ref="D41" r:id="rId47" xr:uid="{9B0CA447-45E8-D346-B56C-D40A5B7E7394}"/>
-    <hyperlink ref="D53" r:id="rId48" xr:uid="{6BBC2247-F5A6-2B4C-BCC0-65AE168D0F4C}"/>
-    <hyperlink ref="D59" r:id="rId49" xr:uid="{08F79F8D-E59F-AA49-A346-A986D8DD0952}"/>
-    <hyperlink ref="D13" r:id="rId50" xr:uid="{7C13DFA2-9F0D-4A4B-8033-EEC7EC90A886}"/>
-    <hyperlink ref="D39" r:id="rId51" xr:uid="{DC9C8D1E-F476-4A4E-902C-35F1A9CEBD2C}"/>
-    <hyperlink ref="D54" r:id="rId52" xr:uid="{EC2CA3F2-625A-A54A-89A9-746E67B059A2}"/>
+    <hyperlink ref="D11" r:id="rId45" xr:uid="{531FF59E-3ED0-7647-A071-9938F307CC65}"/>
+    <hyperlink ref="D34" r:id="rId46" xr:uid="{F44184D1-3BA6-CA4D-B592-38E9B7DD9585}"/>
+    <hyperlink ref="D43" r:id="rId47" xr:uid="{9B0CA447-45E8-D346-B56C-D40A5B7E7394}"/>
+    <hyperlink ref="D55" r:id="rId48" xr:uid="{6BBC2247-F5A6-2B4C-BCC0-65AE168D0F4C}"/>
+    <hyperlink ref="D62" r:id="rId49" xr:uid="{08F79F8D-E59F-AA49-A346-A986D8DD0952}"/>
+    <hyperlink ref="D14" r:id="rId50" xr:uid="{7C13DFA2-9F0D-4A4B-8033-EEC7EC90A886}"/>
+    <hyperlink ref="D41" r:id="rId51" xr:uid="{DC9C8D1E-F476-4A4E-902C-35F1A9CEBD2C}"/>
+    <hyperlink ref="D56" r:id="rId52" xr:uid="{EC2CA3F2-625A-A54A-89A9-746E67B059A2}"/>
+    <hyperlink ref="D10" r:id="rId53" xr:uid="{0A1D472B-DE81-5E43-9A8E-3DA642D15761}"/>
+    <hyperlink ref="D16" r:id="rId54" xr:uid="{B4A339CC-FA33-4B47-BAEE-9C1470667685}"/>
+    <hyperlink ref="D59" r:id="rId55" location="1631294260433-cce691d9-4a8c" xr:uid="{80C75159-965F-8342-ABDD-BA0AF1B41DD0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>